<commit_message>
Update CO - Splunk Intermediate (1).xlsx
</commit_message>
<xml_diff>
--- a/CO - Splunk Intermediate (1).xlsx
+++ b/CO - Splunk Intermediate (1).xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\VK_GIT\SPLK_CISCO_10_12_2025\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CDAD4C60-5C77-419D-9B00-D73851D1A166}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{57AAE29A-AE02-481C-99E6-92F4F6B09028}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -456,7 +456,7 @@
       <charset val="1"/>
     </font>
   </fonts>
-  <fills count="4">
+  <fills count="5">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -475,6 +475,12 @@
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FF92D050"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
   </fills>
   <borders count="11">
     <border>
@@ -602,7 +608,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="26">
+  <cellXfs count="28">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
@@ -619,6 +625,21 @@
       <alignment horizontal="left" vertical="top"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="3" fillId="3" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="3" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="3" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="3" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="3" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="1" fillId="3" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="1" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
@@ -637,24 +658,15 @@
     <xf numFmtId="0" fontId="1" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="3" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="3" fillId="4" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="3" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="4" fillId="4" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="3" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="4" fillId="4" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="3" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="3" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="4" fillId="3" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="3" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="1" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -1003,21 +1015,21 @@
       <c r="A1" s="2" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="15" t="s">
+      <c r="B1" s="22" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="16"/>
-      <c r="D1" s="17"/>
+      <c r="C1" s="23"/>
+      <c r="D1" s="24"/>
     </row>
     <row r="2" spans="1:5" ht="29.25" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A2" s="2" t="s">
         <v>2</v>
       </c>
-      <c r="B2" s="12" t="s">
+      <c r="B2" s="19" t="s">
         <v>3</v>
       </c>
-      <c r="C2" s="13"/>
-      <c r="D2" s="14"/>
+      <c r="C2" s="20"/>
+      <c r="D2" s="21"/>
       <c r="E2" s="11"/>
     </row>
     <row r="4" spans="1:5" x14ac:dyDescent="0.3">
@@ -1036,369 +1048,369 @@
       <c r="A5" s="10" t="s">
         <v>7</v>
       </c>
-      <c r="B5" s="18" t="s">
+      <c r="B5" s="25" t="s">
         <v>8</v>
       </c>
-      <c r="C5" s="19" t="s">
+      <c r="C5" s="13" t="s">
         <v>9</v>
       </c>
-      <c r="D5" s="19" t="s">
+      <c r="D5" s="13" t="s">
         <v>10</v>
       </c>
     </row>
     <row r="6" spans="1:5" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="B6" s="20" t="s">
+      <c r="B6" s="26" t="s">
         <v>11</v>
       </c>
-      <c r="C6" s="21" t="s">
+      <c r="C6" s="15" t="s">
         <v>12</v>
       </c>
-      <c r="D6" s="21" t="s">
+      <c r="D6" s="15" t="s">
         <v>13</v>
       </c>
     </row>
     <row r="7" spans="1:5" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="B7" s="20" t="s">
+      <c r="B7" s="26" t="s">
         <v>14</v>
       </c>
-      <c r="C7" s="21" t="s">
+      <c r="C7" s="15" t="s">
         <v>15</v>
       </c>
-      <c r="D7" s="21" t="s">
+      <c r="D7" s="15" t="s">
         <v>16</v>
       </c>
     </row>
     <row r="8" spans="1:5" ht="31.2" x14ac:dyDescent="0.3">
-      <c r="B8" s="20" t="s">
+      <c r="B8" s="26" t="s">
         <v>17</v>
       </c>
-      <c r="C8" s="21" t="s">
+      <c r="C8" s="15" t="s">
         <v>18</v>
       </c>
-      <c r="D8" s="21" t="s">
+      <c r="D8" s="15" t="s">
         <v>19</v>
       </c>
     </row>
     <row r="9" spans="1:5" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="B9" s="20" t="s">
+      <c r="B9" s="14" t="s">
         <v>20</v>
       </c>
-      <c r="C9" s="21" t="s">
+      <c r="C9" s="15" t="s">
         <v>21</v>
       </c>
-      <c r="D9" s="21" t="s">
+      <c r="D9" s="15" t="s">
         <v>20</v>
       </c>
     </row>
     <row r="10" spans="1:5" ht="31.2" x14ac:dyDescent="0.3">
-      <c r="B10" s="18" t="s">
+      <c r="B10" s="25" t="s">
         <v>22</v>
       </c>
-      <c r="C10" s="21" t="s">
+      <c r="C10" s="15" t="s">
         <v>23</v>
       </c>
-      <c r="D10" s="19" t="s">
+      <c r="D10" s="13" t="s">
         <v>24</v>
       </c>
     </row>
     <row r="11" spans="1:5" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="B11" s="20" t="s">
+      <c r="B11" s="26" t="s">
         <v>25</v>
       </c>
-      <c r="C11" s="21" t="s">
+      <c r="C11" s="15" t="s">
         <v>26</v>
       </c>
-      <c r="D11" s="21" t="s">
+      <c r="D11" s="15" t="s">
         <v>27</v>
       </c>
     </row>
     <row r="12" spans="1:5" ht="31.2" x14ac:dyDescent="0.3">
-      <c r="B12" s="20" t="s">
+      <c r="B12" s="26" t="s">
         <v>28</v>
       </c>
-      <c r="C12" s="21" t="s">
+      <c r="C12" s="15" t="s">
         <v>20</v>
       </c>
-      <c r="D12" s="21" t="s">
+      <c r="D12" s="15" t="s">
         <v>29</v>
       </c>
     </row>
     <row r="13" spans="1:5" ht="31.2" x14ac:dyDescent="0.3">
-      <c r="B13" s="20" t="s">
+      <c r="B13" s="26" t="s">
         <v>30</v>
       </c>
-      <c r="C13" s="19" t="s">
+      <c r="C13" s="13" t="s">
         <v>31</v>
       </c>
-      <c r="D13" s="21" t="s">
+      <c r="D13" s="15" t="s">
         <v>32</v>
       </c>
     </row>
     <row r="14" spans="1:5" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="B14" s="20" t="s">
+      <c r="B14" s="26" t="s">
         <v>33</v>
       </c>
-      <c r="C14" s="21" t="s">
+      <c r="C14" s="15" t="s">
         <v>34</v>
       </c>
-      <c r="D14" s="21" t="s">
+      <c r="D14" s="15" t="s">
         <v>35</v>
       </c>
     </row>
     <row r="15" spans="1:5" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="B15" s="20" t="s">
+      <c r="B15" s="14" t="s">
         <v>20</v>
       </c>
-      <c r="C15" s="21" t="s">
+      <c r="C15" s="15" t="s">
         <v>36</v>
       </c>
-      <c r="D15" s="21" t="s">
+      <c r="D15" s="15" t="s">
         <v>37</v>
       </c>
     </row>
     <row r="16" spans="1:5" ht="31.2" x14ac:dyDescent="0.3">
-      <c r="B16" s="18" t="s">
+      <c r="B16" s="12" t="s">
         <v>38</v>
       </c>
-      <c r="C16" s="21" t="s">
+      <c r="C16" s="15" t="s">
         <v>39</v>
       </c>
-      <c r="D16" s="21" t="s">
+      <c r="D16" s="15" t="s">
         <v>20</v>
       </c>
     </row>
     <row r="17" spans="2:4" ht="31.2" x14ac:dyDescent="0.3">
-      <c r="B17" s="20" t="s">
+      <c r="B17" s="26" t="s">
         <v>40</v>
       </c>
-      <c r="C17" s="21" t="s">
+      <c r="C17" s="15" t="s">
         <v>20</v>
       </c>
-      <c r="D17" s="19" t="s">
+      <c r="D17" s="13" t="s">
         <v>41</v>
       </c>
     </row>
     <row r="18" spans="2:4" ht="31.2" x14ac:dyDescent="0.3">
-      <c r="B18" s="20" t="s">
+      <c r="B18" s="26" t="s">
         <v>42</v>
       </c>
-      <c r="C18" s="19" t="s">
+      <c r="C18" s="13" t="s">
         <v>43</v>
       </c>
-      <c r="D18" s="21" t="s">
+      <c r="D18" s="15" t="s">
         <v>44</v>
       </c>
     </row>
     <row r="19" spans="2:4" ht="31.2" x14ac:dyDescent="0.3">
-      <c r="B19" s="20" t="s">
+      <c r="B19" s="26" t="s">
         <v>45</v>
       </c>
-      <c r="C19" s="21" t="s">
+      <c r="C19" s="15" t="s">
         <v>46</v>
       </c>
-      <c r="D19" s="21" t="s">
+      <c r="D19" s="15" t="s">
         <v>47</v>
       </c>
     </row>
     <row r="20" spans="2:4" ht="31.2" x14ac:dyDescent="0.3">
-      <c r="B20" s="20" t="s">
+      <c r="B20" s="26" t="s">
         <v>48</v>
       </c>
-      <c r="C20" s="21" t="s">
+      <c r="C20" s="15" t="s">
         <v>49</v>
       </c>
-      <c r="D20" s="21" t="s">
+      <c r="D20" s="15" t="s">
         <v>50</v>
       </c>
     </row>
     <row r="21" spans="2:4" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="B21" s="20" t="s">
+      <c r="B21" s="14" t="s">
         <v>20</v>
       </c>
-      <c r="C21" s="21" t="s">
+      <c r="C21" s="15" t="s">
         <v>20</v>
       </c>
-      <c r="D21" s="22"/>
+      <c r="D21" s="16"/>
     </row>
     <row r="22" spans="2:4" ht="31.2" x14ac:dyDescent="0.3">
-      <c r="B22" s="18" t="s">
+      <c r="B22" s="12" t="s">
         <v>51</v>
       </c>
-      <c r="C22" s="19" t="s">
+      <c r="C22" s="13" t="s">
         <v>52</v>
       </c>
-      <c r="D22" s="22"/>
+      <c r="D22" s="16"/>
     </row>
     <row r="23" spans="2:4" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="B23" s="20" t="s">
+      <c r="B23" s="14" t="s">
         <v>53</v>
       </c>
-      <c r="C23" s="21" t="s">
+      <c r="C23" s="15" t="s">
         <v>54</v>
       </c>
-      <c r="D23" s="22"/>
+      <c r="D23" s="16"/>
     </row>
     <row r="24" spans="2:4" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="B24" s="20" t="s">
+      <c r="B24" s="14" t="s">
         <v>55</v>
       </c>
-      <c r="C24" s="21" t="s">
+      <c r="C24" s="15" t="s">
         <v>56</v>
       </c>
-      <c r="D24" s="22"/>
+      <c r="D24" s="16"/>
     </row>
     <row r="25" spans="2:4" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="B25" s="20" t="s">
+      <c r="B25" s="14" t="s">
         <v>57</v>
       </c>
-      <c r="C25" s="21" t="s">
+      <c r="C25" s="15" t="s">
         <v>58</v>
       </c>
-      <c r="D25" s="22"/>
+      <c r="D25" s="16"/>
     </row>
     <row r="26" spans="2:4" ht="31.2" x14ac:dyDescent="0.3">
-      <c r="B26" s="20" t="s">
+      <c r="B26" s="26" t="s">
         <v>59</v>
       </c>
-      <c r="C26" s="21" t="s">
+      <c r="C26" s="15" t="s">
         <v>20</v>
       </c>
-      <c r="D26" s="22"/>
+      <c r="D26" s="16"/>
     </row>
     <row r="27" spans="2:4" ht="31.2" x14ac:dyDescent="0.3">
-      <c r="B27" s="20" t="s">
+      <c r="B27" s="26" t="s">
         <v>60</v>
       </c>
-      <c r="C27" s="19" t="s">
+      <c r="C27" s="13" t="s">
         <v>61</v>
       </c>
-      <c r="D27" s="22"/>
+      <c r="D27" s="16"/>
     </row>
     <row r="28" spans="2:4" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="B28" s="20" t="s">
+      <c r="B28" s="26" t="s">
         <v>62</v>
       </c>
-      <c r="C28" s="21" t="s">
+      <c r="C28" s="15" t="s">
         <v>63</v>
       </c>
-      <c r="D28" s="22"/>
+      <c r="D28" s="16"/>
     </row>
     <row r="29" spans="2:4" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="B29" s="20" t="s">
+      <c r="B29" s="26" t="s">
         <v>64</v>
       </c>
-      <c r="C29" s="21" t="s">
+      <c r="C29" s="15" t="s">
         <v>65</v>
       </c>
-      <c r="D29" s="22"/>
+      <c r="D29" s="16"/>
     </row>
     <row r="30" spans="2:4" ht="31.2" x14ac:dyDescent="0.3">
-      <c r="B30" s="20" t="s">
+      <c r="B30" s="26" t="s">
         <v>66</v>
       </c>
-      <c r="C30" s="21" t="s">
+      <c r="C30" s="15" t="s">
         <v>67</v>
       </c>
-      <c r="D30" s="22"/>
+      <c r="D30" s="16"/>
     </row>
     <row r="31" spans="2:4" ht="31.2" x14ac:dyDescent="0.3">
-      <c r="B31" s="18" t="s">
+      <c r="B31" s="12" t="s">
         <v>68</v>
       </c>
-      <c r="C31" s="21" t="s">
+      <c r="C31" s="15" t="s">
         <v>69</v>
       </c>
-      <c r="D31" s="22"/>
+      <c r="D31" s="16"/>
     </row>
     <row r="32" spans="2:4" ht="31.2" x14ac:dyDescent="0.3">
-      <c r="B32" s="20" t="s">
+      <c r="B32" s="14" t="s">
         <v>70</v>
       </c>
-      <c r="C32" s="22"/>
-      <c r="D32" s="22"/>
+      <c r="C32" s="16"/>
+      <c r="D32" s="16"/>
     </row>
     <row r="33" spans="1:4" ht="46.8" x14ac:dyDescent="0.3">
-      <c r="B33" s="20" t="s">
+      <c r="B33" s="14" t="s">
         <v>71</v>
       </c>
-      <c r="C33" s="22"/>
-      <c r="D33" s="22"/>
+      <c r="C33" s="16"/>
+      <c r="D33" s="16"/>
     </row>
     <row r="34" spans="1:4" ht="46.8" x14ac:dyDescent="0.3">
-      <c r="B34" s="20" t="s">
+      <c r="B34" s="14" t="s">
         <v>72</v>
       </c>
-      <c r="C34" s="22"/>
-      <c r="D34" s="22"/>
+      <c r="C34" s="16"/>
+      <c r="D34" s="16"/>
     </row>
     <row r="35" spans="1:4" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="B35" s="20" t="s">
+      <c r="B35" s="14" t="s">
         <v>20</v>
       </c>
-      <c r="C35" s="22"/>
-      <c r="D35" s="22"/>
+      <c r="C35" s="16"/>
+      <c r="D35" s="16"/>
     </row>
     <row r="36" spans="1:4" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="B36" s="20" t="s">
+      <c r="B36" s="14" t="s">
         <v>20</v>
       </c>
-      <c r="C36" s="22"/>
-      <c r="D36" s="22"/>
+      <c r="C36" s="16"/>
+      <c r="D36" s="16"/>
     </row>
     <row r="37" spans="1:4" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="B37" s="18" t="s">
+      <c r="B37" s="25" t="s">
         <v>73</v>
       </c>
-      <c r="C37" s="22"/>
-      <c r="D37" s="22"/>
+      <c r="C37" s="16"/>
+      <c r="D37" s="16"/>
     </row>
     <row r="38" spans="1:4" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="B38" s="20" t="s">
+      <c r="B38" s="26" t="s">
         <v>74</v>
       </c>
-      <c r="C38" s="22"/>
-      <c r="D38" s="22"/>
+      <c r="C38" s="16"/>
+      <c r="D38" s="16"/>
     </row>
     <row r="39" spans="1:4" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="B39" s="20" t="s">
+      <c r="B39" s="26" t="s">
         <v>75</v>
       </c>
-      <c r="C39" s="22"/>
-      <c r="D39" s="22"/>
+      <c r="C39" s="16"/>
+      <c r="D39" s="16"/>
     </row>
     <row r="40" spans="1:4" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="B40" s="20" t="s">
+      <c r="B40" s="26" t="s">
         <v>76</v>
       </c>
-      <c r="C40" s="22"/>
-      <c r="D40" s="22"/>
+      <c r="C40" s="16"/>
+      <c r="D40" s="16"/>
     </row>
     <row r="41" spans="1:4" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="B41" s="20" t="s">
+      <c r="B41" s="26" t="s">
         <v>77</v>
       </c>
-      <c r="C41" s="22"/>
-      <c r="D41" s="22"/>
+      <c r="C41" s="16"/>
+      <c r="D41" s="16"/>
     </row>
     <row r="42" spans="1:4" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="B42" s="20" t="s">
+      <c r="B42" s="26" t="s">
         <v>78</v>
       </c>
-      <c r="C42" s="22"/>
-      <c r="D42" s="22"/>
+      <c r="C42" s="16"/>
+      <c r="D42" s="16"/>
     </row>
     <row r="43" spans="1:4" ht="31.2" x14ac:dyDescent="0.3">
       <c r="A43" s="4"/>
-      <c r="B43" s="23" t="s">
+      <c r="B43" s="27" t="s">
         <v>79</v>
       </c>
-      <c r="C43" s="24"/>
-      <c r="D43" s="24"/>
+      <c r="C43" s="17"/>
+      <c r="D43" s="17"/>
     </row>
     <row r="44" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="B44" s="25"/>
-      <c r="C44" s="25"/>
-      <c r="D44" s="25"/>
+      <c r="B44" s="18"/>
+      <c r="C44" s="18"/>
+      <c r="D44" s="18"/>
     </row>
     <row r="45" spans="1:4" ht="18" x14ac:dyDescent="0.35">
       <c r="A45" s="7" t="s">
@@ -1422,26 +1434,6 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
-</file>
-
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement>
-    <lcf76f155ced4ddcb4097134ff3c332f xmlns="ac015f5f-37cf-480b-8f61-9f6dcabe93df">
-      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    </lcf76f155ced4ddcb4097134ff3c332f>
-    <TaxCatchAll xmlns="5b6e755b-8d33-4086-9b6b-a9a4d44f3067" xsi:nil="true"/>
-  </documentManagement>
-</p:properties>
-</file>
-
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x0101001AF7E30AC51BE24AB98F695D1F646B0D" ma:contentTypeVersion="15" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="944c3efe05a27205f6f8a21900784054">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="ac015f5f-37cf-480b-8f61-9f6dcabe93df" xmlns:ns3="5b6e755b-8d33-4086-9b6b-a9a4d44f3067" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="0bdc8c47fb571a171e530ebc6f1b62f9" ns2:_="" ns3:_="">
     <xsd:import namespace="ac015f5f-37cf-480b-8f61-9f6dcabe93df"/>
@@ -1676,10 +1668,41 @@
 </ct:contentTypeSchema>
 </file>
 
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement>
+    <lcf76f155ced4ddcb4097134ff3c332f xmlns="ac015f5f-37cf-480b-8f61-9f6dcabe93df">
+      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    </lcf76f155ced4ddcb4097134ff3c332f>
+    <TaxCatchAll xmlns="5b6e755b-8d33-4086-9b6b-a9a4d44f3067" xsi:nil="true"/>
+  </documentManagement>
+</p:properties>
+</file>
+
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
+</file>
+
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{B3C898FD-DFB1-448F-9432-BD9DD563A099}">
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{889D0D1E-5983-4BD8-861A-9A522ED044AD}">
   <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes"/>
+    <ds:schemaRef ds:uri="http://www.w3.org/2001/XMLSchema"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="ac015f5f-37cf-480b-8f61-9f6dcabe93df"/>
+    <ds:schemaRef ds:uri="5b6e755b-8d33-4086-9b6b-a9a4d44f3067"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/internal/obd"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
 </file>
@@ -1696,20 +1719,9 @@
 </file>
 
 <file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{889D0D1E-5983-4BD8-861A-9A522ED044AD}">
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{B3C898FD-DFB1-448F-9432-BD9DD563A099}">
   <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes"/>
-    <ds:schemaRef ds:uri="http://www.w3.org/2001/XMLSchema"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
-    <ds:schemaRef ds:uri="ac015f5f-37cf-480b-8f61-9f6dcabe93df"/>
-    <ds:schemaRef ds:uri="5b6e755b-8d33-4086-9b6b-a9a4d44f3067"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/internal/obd"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
 </file>
</xml_diff>